<commit_message>
Correo de Jhoan: version corta queda como la unica en RESPUESTA_TRASLADO_BOGOTA.xlsx; eliminado el archivo auxiliar
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/recursos/experiencia_cliente/RESPUESTA_TRASLADO_BOGOTA.xlsx
+++ b/recursos/experiencia_cliente/RESPUESTA_TRASLADO_BOGOTA.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RESPUESTA TRASLADO BOGOTA" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CORREO JHOAN" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A24"/>
+  <dimension ref="A1:A18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -429,7 +429,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Buenas tardes, [nombre del acudiente]:</t>
+          <t>Buenas tardes:</t>
         </is>
       </c>
     </row>
@@ -439,7 +439,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Gracias por escribirnos y por contarnos su situación con tiempo. Lo primero: felicitaciones a [nombre del estudiante] — su compromiso y su nivel son exactamente lo que nos confirman sus profesores. Y le tenemos la noticia que esperaban: su nota del nivel A2 es [NOTA], nivel aprobado. Su certificado queda disponible.</t>
+          <t>Gracias por escribirnos con tiempo. Lo primero: felicitaciones a Jhoan — su compromiso es el que nos confirman sus profesores, y su nota del A2 es [NOTA]: nivel aprobado, certificado disponible.</t>
         </is>
       </c>
     </row>
@@ -449,7 +449,7 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>Ahora, sobre su solicitud — queremos ayudarles a que avance lo máximo posible antes del viaje, y esta es nuestra propuesta, SIN COSTO ADICIONAL para ustedes:</t>
+          <t>Nuestra propuesta para que avance lo máximo antes del viaje, SIN COSTO ADICIONAL: mientras estén en la ciudad, Jhoan cursa el B1 en DOBLE JORNADA — sigue en su grupo de la noche y además entra al B1 intensivo de 4 horas que abre el miércoles 30 de septiembre. Doble velocidad.</t>
         </is>
       </c>
     </row>
@@ -459,21 +459,17 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>Mientras estén en la ciudad, [nombre] avanza el nivel B1 en DOBLE JORNADA:</t>
+          <t>Una claridad para que la experiencia sea la correcta: habrá temas repetidos entre las dos jornadas, y en B1 el avance se siente más lento que en los primeros niveles — es como un nadador: para bajar un segundo hay que nadar miles de piscinas. Esa repetición es el entrenamiento que fija el idioma, es la parte más difícil del camino, y el que la atraviesa es el que persevera. Jhoan es de esos.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>· Continúa en su grupo B1 de la noche, como hasta ahora.</t>
-        </is>
-      </c>
+      <c r="A8" s="1" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>· Y ADEMÁS se adelanta en el B1 intensivo de 4 horas diarias que abre el miércoles 30 de septiembre. Asistiendo a ambas jornadas, cubre el nivel a más del doble de velocidad.</t>
+          <t>Para armarle el plan exacto solo necesitamos un dato: ¿PARA QUÉ FECHA tienen previsto el viaje?</t>
         </is>
       </c>
     </row>
@@ -483,7 +479,7 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>Una claridad importante para que la experiencia sea la correcta: al ver el mismo nivel en dos jornadas, habrá temas que se repitan, y en B1 (igual que después en B2) la sensación de avance es distinta a los primeros niveles — se avanza más profundo y menos "visible". Es como un nadador: para bajar un solo segundo hay que nadar miles de piscinas. Esa repetición no es tiempo perdido: es el entrenamiento que fija el idioma — y es la parte más difícil del camino. El que la atraviesa es el que persevera, y por lo que conocemos de [nombre del estudiante], él es de esos.</t>
+          <t>Sobre Zoom, con honestidad: nuestro método es presencial — es la razón por la que Jhoan ha avanzado así — y no dictamos niveles virtuales. Por eso la propuesta es aprovechar al máximo el tiempo presencial y entregarle sus certificados oficiales de todo lo que apruebe, válidos en cualquier ciudad.</t>
         </is>
       </c>
     </row>
@@ -493,7 +489,7 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>Para armarle el plan exacto necesitamos un dato: ¿PARA QUÉ FECHA tienen previsto el viaje? Con esa fecha calculamos hasta dónde alcanza a llegar y coordinamos su evaluación con el equipo académico.</t>
+          <t>Un único favor a cambio: cuando el plan esté andando, regálennos un testimonio corto en video de la experiencia de Jhoan. Familias como ustedes son nuestra mejor carta de presentación.</t>
         </is>
       </c>
     </row>
@@ -503,7 +499,7 @@
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>Sobre la opción por Zoom, con total honestidad: nuestro método es presencial — es la razón por la que [nombre] ha avanzado como ha avanzado — y no ofrecemos los niveles de forma virtual. Por eso preferimos que aproveche al máximo el tiempo presencial que les queda, y entregarle sus certificados oficiales de todo lo que curse y apruebe, que le sirven en cualquier ciudad.</t>
+          <t>Sus cuotas siguen su calendario normal. Quedamos atentos a la fecha para dejar todo andando esta semana.</t>
         </is>
       </c>
     </row>
@@ -513,42 +509,12 @@
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>Y un único favor a cambio, que para nosotros vale oro: cuando el plan esté andando, regálennos un testimonio corto en video de la experiencia de [nombre] en la academia. Familias como ustedes son la mejor carta de presentación que tenemos.</t>
+          <t>Cordialmente,</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="1" t="inlineStr">
-        <is>
-          <t>Sus cuotas pendientes continúan con su calendario normal, sin ningún cambio.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="1" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="1" t="inlineStr">
-        <is>
-          <t>Quedamos atentos a la fecha del viaje para dejar el plan andando esta misma semana.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="1" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="1" t="inlineStr">
-        <is>
-          <t>Cordialmente,</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="1" t="inlineStr">
+      <c r="A18" s="1" t="inlineStr">
         <is>
           <t>Depto. Experiencia al Cliente — Heiiu English Academy</t>
         </is>

</xml_diff>